<commit_message>
chore: resolve locks before merge
</commit_message>
<xml_diff>
--- a/Stock and dividend overview_3Mar2026.xlsx
+++ b/Stock and dividend overview_3Mar2026.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Paulo\Projects\investment-advisor\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8E8CA4CB-D8E9-4A70-991A-715FF5FD9310}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F3074C1E-E2EC-4352-9AA5-8D557651C475}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="51840" windowHeight="21240" xr2:uid="{9A434641-3564-486F-B303-B8171EC270D7}"/>
   </bookViews>
@@ -26001,7 +26001,7 @@
       </c>
       <c r="U16" s="16"/>
     </row>
-    <row r="17" spans="1:16384" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:16384" x14ac:dyDescent="0.25">
       <c r="A17" s="137">
         <v>16</v>
       </c>
@@ -26064,7 +26064,7 @@
       </c>
       <c r="U17" s="16"/>
     </row>
-    <row r="18" spans="1:16384" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:16384" x14ac:dyDescent="0.25">
       <c r="A18" s="137">
         <v>17</v>
       </c>
@@ -26125,7 +26125,7 @@
       </c>
       <c r="U18" s="16"/>
     </row>
-    <row r="19" spans="1:16384" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:16384" x14ac:dyDescent="0.25">
       <c r="A19" s="137">
         <v>18</v>
       </c>
@@ -42610,7 +42610,7 @@
       <c r="XFC20"/>
       <c r="XFD20" s="1"/>
     </row>
-    <row r="21" spans="1:16384" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:16384" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A21" s="144">
         <v>20</v>
       </c>
@@ -42669,7 +42669,7 @@
       </c>
       <c r="U21" s="17"/>
     </row>
-    <row r="22" spans="1:16384" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:16384" x14ac:dyDescent="0.25">
       <c r="A22" s="132">
         <v>1</v>
       </c>
@@ -42736,7 +42736,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="23" spans="1:16384" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:16384" x14ac:dyDescent="0.25">
       <c r="A23" s="137">
         <v>2</v>
       </c>
@@ -42797,7 +42797,7 @@
       </c>
       <c r="U23" s="16"/>
     </row>
-    <row r="24" spans="1:16384" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:16384" x14ac:dyDescent="0.25">
       <c r="A24" s="137">
         <v>3</v>
       </c>
@@ -42860,7 +42860,7 @@
       </c>
       <c r="U24" s="16"/>
     </row>
-    <row r="25" spans="1:16384" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:16384" x14ac:dyDescent="0.25">
       <c r="A25" s="137">
         <v>4</v>
       </c>
@@ -42921,7 +42921,7 @@
       </c>
       <c r="U25" s="16"/>
     </row>
-    <row r="26" spans="1:16384" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:16384" x14ac:dyDescent="0.25">
       <c r="A26" s="137">
         <v>5</v>
       </c>
@@ -42983,7 +42983,7 @@
       </c>
       <c r="U26" s="16"/>
     </row>
-    <row r="27" spans="1:16384" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:16384" x14ac:dyDescent="0.25">
       <c r="A27" s="137">
         <v>6</v>
       </c>
@@ -43044,7 +43044,7 @@
       </c>
       <c r="U27" s="16"/>
     </row>
-    <row r="28" spans="1:16384" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:16384" x14ac:dyDescent="0.25">
       <c r="A28" s="137">
         <v>7</v>
       </c>
@@ -43105,7 +43105,7 @@
       </c>
       <c r="U28" s="16"/>
     </row>
-    <row r="29" spans="1:16384" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:16384" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A29" s="144">
         <v>8</v>
       </c>
@@ -43166,7 +43166,7 @@
       </c>
       <c r="U29" s="17"/>
     </row>
-    <row r="30" spans="1:16384" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:16384" x14ac:dyDescent="0.25">
       <c r="A30" s="150"/>
       <c r="B30" s="167" t="s">
         <v>109</v>
@@ -43227,7 +43227,7 @@
       </c>
       <c r="U30" s="11"/>
     </row>
-    <row r="31" spans="1:16384" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:16384" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A31" s="13"/>
       <c r="B31" s="169" t="s">
         <v>109</v>
@@ -43288,7 +43288,7 @@
       </c>
       <c r="U31" s="17"/>
     </row>
-    <row r="32" spans="1:16384" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:16384" x14ac:dyDescent="0.25">
       <c r="A32" s="12"/>
       <c r="B32" s="168" t="s">
         <v>128</v>

</xml_diff>